<commit_message>
Unidad 1: contenido faltante (prestaciones), fix de tope Art. 58 en Excel, emojis por íconos SVG y 3 diagramas nuevos
</commit_message>
<xml_diff>
--- a/Entregables/Unidad 1/U1_Planillas_ContFinanciera.xlsx
+++ b/Entregables/Unidad 1/U1_Planillas_ContFinanciera.xlsx
@@ -173,7 +173,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -318,11 +318,80 @@
         <color rgb="001E2D5A"/>
       </top>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00F9A825"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEEC"/>
+      </right>
+      <top style="medium">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEEC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00F9A825"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D9DEEC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D9DEEC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEEC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D9DEEC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -400,6 +469,13 @@
     <xf numFmtId="164" fontId="10" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="10" fillId="9" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -883,27 +959,23 @@
           <t>"Por mi honor y ante mis compañeros, me comprometo a que esta actividad académica refleje mi verdadero nivel de conocimientos, evitando realizar cualquier forma de deshonestidad académica (por ejemplo, copiar o plagiar)."</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="10" t="n"/>
+      <c r="C12" s="59" t="n"/>
+      <c r="D12" s="59" t="n"/>
+      <c r="E12" s="60" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="13" t="n"/>
+      <c r="B13" s="61" t="n"/>
+      <c r="E13" s="62" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="13" t="n"/>
+      <c r="B14" s="61" t="n"/>
+      <c r="E14" s="62" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="15" t="n"/>
-      <c r="E15" s="16" t="n"/>
+      <c r="B15" s="63" t="n"/>
+      <c r="C15" s="64" t="n"/>
+      <c r="D15" s="64" t="n"/>
+      <c r="E15" s="65" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
@@ -1154,7 +1226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G65"/>
+  <dimension ref="B2:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2091,6 +2163,13 @@
       <c r="B65" s="39" t="inlineStr">
         <is>
           <t>• Aguinaldo: exento de ISR hasta el equivalente a 2 salarios mínimos mensuales del sector comercio y servicios; el exceso se grava con la tabla mensual de ISR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>• Indemnización por despido incausado: para el cálculo del monto (30 días de salario básico por año), ningún salario diario puede considerarse superior a 4 veces el salario mínimo diario legal vigente — Art. 58, Código de Trabajo.</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3822,7 @@
         <v/>
       </c>
       <c r="L5" s="40">
-        <f>ROUND(C5*D5,2)</f>
+        <f>ROUND(MIN(E5,ROUND(('2. Marco Normativo'!$C$48*4)/30,2))*30*D5,2)</f>
         <v/>
       </c>
       <c r="M5" s="40">
@@ -3752,7 +3831,7 @@
       </c>
       <c r="N5" s="41" t="inlineStr">
         <is>
-          <t>4 años de antigüedad → tabla de aguinaldo: 3-10 años = 19 días. Aguinaldo bajo el tope exento (2 SM), no paga ISR.</t>
+          <t>4 años de antigüedad → tabla de aguinaldo: 3-10 años = 19 días. Aguinaldo bajo el tope exento (2 SM), no paga ISR. Indemnización con salario diario topado a 4 salarios mínimos diarios (Art. 58, Código de Trabajo).</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3876,7 @@
         <v/>
       </c>
       <c r="L6" s="40">
-        <f>ROUND(C6*D6,2)</f>
+        <f>ROUND(MIN(E6,ROUND(('2. Marco Normativo'!$C$48*4)/30,2))*30*D6,2)</f>
         <v/>
       </c>
       <c r="M6" s="40">
@@ -3806,7 +3885,7 @@
       </c>
       <c r="N6" s="41" t="inlineStr">
         <is>
-          <t>12 años de antigüedad → 10+ años = 21 días. Aguinaldo supera el tope exento; el exceso paga ISR y la renuncia voluntaria se topa a 2 salarios mínimos diarios.</t>
+          <t>12 años de antigüedad → 10+ años = 21 días. Aguinaldo supera el tope exento; el exceso paga ISR. Su salario diario ($83.33) supera el tope de 4 salarios mínimos diarios ($54.51), así que la indemnización se calcula con el tope, no con su salario real — y la renuncia voluntaria se topa a 2 salarios mínimos diarios.</t>
         </is>
       </c>
     </row>
@@ -3973,7 +4052,7 @@
         <v/>
       </c>
       <c r="L5" s="40">
-        <f>ROUND(C5*D5,2)</f>
+        <f>ROUND(MIN(E5,ROUND(('2. Marco Normativo'!$C$48*4)/30,2))*30*D5,2)</f>
         <v/>
       </c>
       <c r="M5" s="40">
@@ -4025,7 +4104,7 @@
         <v/>
       </c>
       <c r="L6" s="40">
-        <f>ROUND(C6*D6,2)</f>
+        <f>ROUND(MIN(E6,ROUND(('2. Marco Normativo'!$C$48*4)/30,2))*30*D6,2)</f>
         <v/>
       </c>
       <c r="M6" s="40">
@@ -4077,7 +4156,7 @@
         <v/>
       </c>
       <c r="L7" s="40">
-        <f>ROUND(C7*D7,2)</f>
+        <f>ROUND(MIN(E7,ROUND(('2. Marco Normativo'!$C$48*4)/30,2))*30*D7,2)</f>
         <v/>
       </c>
       <c r="M7" s="40">

</xml_diff>